<commit_message>
Update example test file UsingTables
Update reference test file for example UsingTables. After the style
infrastructure switch, the styles part is saved differently. No semantic
change to the styles part. Many styles were not used and were removed
in new version.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/Tables/UsingTables.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/Tables/UsingTables.xlsx
@@ -73,363 +73,58 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
-    <x:numFmt numFmtId="0" formatCode=""/>
-    <x:numFmt numFmtId="164" formatCode="$ #,##0"/>
-  </x:numFmts>
-  <x:fonts count="2">
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="4">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF6495ED"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF00FFFF"/>
-      </x:patternFill>
-    </x:fill>
-  </x:fills>
-  <x:borders count="10">
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="none">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="thick">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="thick">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="thick">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="thick">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="thick">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="thick">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="thick">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="thick">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="thick">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="thick">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="thick">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="thick">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="18">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="3" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="4" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="5" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="6" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="15" fontId="0" fillId="0" borderId="5" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="6" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="15" fontId="0" fillId="0" borderId="8" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="9" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="15" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="2" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="18">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="15" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="15" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-  <x:dxfs count="3">
-    <x:dxf>
-      <x:numFmt numFmtId="15" formatCode="d-MMM-yy"/>
-    </x:dxf>
-    <x:dxf>
-      <x:numFmt numFmtId="164" formatCode="$ #,##0"/>
-    </x:dxf>
-    <x:dxf>
-      <x:numFmt numFmtId="2" formatCode="0.00"/>
-    </x:dxf>
-  </x:dxfs>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$ #,##0"/>
+  </numFmts>
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -439,9 +134,9 @@
     <x:tableColumn id="1" name="FName" totalsRowLabel="Sum Of Income"/>
     <x:tableColumn id="2" name="LName"/>
     <x:tableColumn id="3" name="Outcast"/>
-    <x:tableColumn id="4" name="DOB" dataDxfId="0"/>
-    <x:tableColumn id="5" name="Income" totalsRowFunction="sum" dataDxfId="1"/>
-    <x:tableColumn id="6" name="Age" totalsRowFunction="average" dataDxfId="2">
+    <x:tableColumn id="4" name="DOB"/>
+    <x:tableColumn id="5" name="Income" totalsRowFunction="sum"/>
+    <x:tableColumn id="6" name="Age" totalsRowFunction="average">
       <x:calculatedColumnFormula>(DATE(2017, 10, 3) - E3) / 365</x:calculatedColumnFormula>
     </x:tableColumn>
   </x:tableColumns>
@@ -783,10 +478,10 @@
       <x:c r="D2" s="0" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E2" s="15" t="s">
+      <x:c r="E2" s="1" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="F2" s="16" t="s">
+      <x:c r="F2" s="2" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
@@ -809,13 +504,13 @@
       <x:c r="D3" s="0" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E3" s="15">
+      <x:c r="E3" s="1">
         <x:v>6961</x:v>
       </x:c>
-      <x:c r="F3" s="16">
+      <x:c r="F3" s="2">
         <x:v>2000</x:v>
       </x:c>
-      <x:c r="G3" s="17">
+      <x:c r="G3" s="3">
         <x:f>(DATE(2017, 10, 3) - E3) / 365</x:f>
       </x:c>
       <x:c r="I3" s="0" t="s">
@@ -835,13 +530,13 @@
       <x:c r="D4" s="0" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E4" s="15">
+      <x:c r="E4" s="1">
         <x:v>2620</x:v>
       </x:c>
-      <x:c r="F4" s="16">
+      <x:c r="F4" s="2">
         <x:v>40000</x:v>
       </x:c>
-      <x:c r="G4" s="17">
+      <x:c r="G4" s="3">
         <x:f>(DATE(2017, 10, 3) - E4) / 365</x:f>
       </x:c>
       <x:c r="I4" s="0" t="s">
@@ -861,13 +556,13 @@
       <x:c r="D5" s="0" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E5" s="15">
+      <x:c r="E5" s="1">
         <x:v>8020</x:v>
       </x:c>
-      <x:c r="F5" s="16">
+      <x:c r="F5" s="2">
         <x:v>10000</x:v>
       </x:c>
-      <x:c r="G5" s="17">
+      <x:c r="G5" s="3">
         <x:f>(DATE(2017, 10, 3) - E5) / 365</x:f>
       </x:c>
       <x:c r="I5" s="0" t="s">
@@ -881,11 +576,11 @@
       <x:c r="B6" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="E6" s="15"/>
-      <x:c r="F6" s="16">
+      <x:c r="E6" s="1"/>
+      <x:c r="F6" s="2">
         <x:f>SUBTOTAL(109,[Income])</x:f>
       </x:c>
-      <x:c r="G6" s="17">
+      <x:c r="G6" s="3">
         <x:f>SUBTOTAL(101,[Age])</x:f>
       </x:c>
       <x:c r="I6" s="0" t="s">

</xml_diff>